<commit_message>
Fix CI: ruff lint errors and pyproject.toml configuration
- Configure ruff to ignore BLE001, SIM102, S110, S112, PLW1510
  (intentional patterns in data pipeline code)
- Exclude notebooks from ruff lint checks
- Fix unused imports in tests/__init__.py
- Fix notebook BOM encoding issue
- Auto-fix import sorting across all scripts
- Add nepse_index_2020_2025.csv data file

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/DATA/02_bank_ratios.xlsx
+++ b/DATA/02_bank_ratios.xlsx
@@ -3918,12 +3918,24 @@
       <c r="M58" t="n">
         <v>34.79023776487428</v>
       </c>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
+      <c r="N58" t="n">
+        <v>118.2692835820896</v>
+      </c>
+      <c r="O58" t="n">
+        <v>73.74696019900499</v>
+      </c>
+      <c r="P58" t="n">
+        <v>94.92859203980099</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>1.723004975124378</v>
+      </c>
+      <c r="R58" t="n">
+        <v>1997.657647058824</v>
+      </c>
+      <c r="S58" t="n">
+        <v>0.74</v>
+      </c>
       <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="n">
@@ -3980,12 +3992,24 @@
       <c r="M59" t="n">
         <v>9.029001728182235</v>
       </c>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
+      <c r="N59" t="n">
+        <v>134.3796029547553</v>
+      </c>
+      <c r="O59" t="n">
+        <v>91.42263157894737</v>
+      </c>
+      <c r="P59" t="n">
+        <v>103.1738088642659</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>2.09028162511542</v>
+      </c>
+      <c r="R59" t="n">
+        <v>2156.046074074074</v>
+      </c>
+      <c r="S59" t="n">
+        <v>0.84</v>
+      </c>
       <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="n">
@@ -4042,13 +4066,23 @@
       <c r="M60" t="n">
         <v>8.923427439844437</v>
       </c>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
+      <c r="N60" t="n">
+        <v>187.8380760626398</v>
+      </c>
+      <c r="O60" t="n">
+        <v>134.3202013422819</v>
+      </c>
+      <c r="P60" t="n">
+        <v>145.9607651006712</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>1.904259507829978</v>
+      </c>
+      <c r="R60" t="n">
+        <v>1817.394372294372</v>
+      </c>
       <c r="S60" t="n">
-        <v>4.5</v>
+        <v>1.62</v>
       </c>
       <c r="T60" t="n">
         <v>2.02</v>
@@ -4110,13 +4144,23 @@
       <c r="M61" t="n">
         <v>7.111801675652793</v>
       </c>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
+      <c r="N61" t="n">
+        <v>200.1678660565724</v>
+      </c>
+      <c r="O61" t="n">
+        <v>137.7384234608985</v>
+      </c>
+      <c r="P61" t="n">
+        <v>165.0763311148087</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>2.664284525790349</v>
+      </c>
+      <c r="R61" t="n">
+        <v>1956.111991869919</v>
+      </c>
       <c r="S61" t="n">
-        <v>3.99</v>
+        <v>3.39</v>
       </c>
       <c r="T61" t="n">
         <v>1.8</v>
@@ -4178,13 +4222,23 @@
       <c r="M62" t="n">
         <v>8.297967245915586</v>
       </c>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
+      <c r="N62" t="n">
+        <v>231.7054450915142</v>
+      </c>
+      <c r="O62" t="n">
+        <v>160.4509567387687</v>
+      </c>
+      <c r="P62" t="n">
+        <v>192.220224625624</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>2.577832778702163</v>
+      </c>
+      <c r="R62" t="n">
+        <v>2094.059736842105</v>
+      </c>
       <c r="S62" t="n">
-        <v>3.6</v>
+        <v>4.45</v>
       </c>
       <c r="T62" t="n">
         <v>1.62</v>
@@ -4246,15 +4300,29 @@
       <c r="M63" t="n">
         <v>8.378398964125218</v>
       </c>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
+      <c r="N63" t="n">
+        <v>265.1071482098251</v>
+      </c>
+      <c r="O63" t="n">
+        <v>171.1040965861782</v>
+      </c>
+      <c r="P63" t="n">
+        <v>218.4121398834305</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>2.465503746877602</v>
+      </c>
+      <c r="R63" t="n">
+        <v>2376.072276119403</v>
+      </c>
+      <c r="S63" t="n">
+        <v>4.48</v>
+      </c>
       <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr"/>
+      <c r="V63" t="n">
+        <v>11.81</v>
+      </c>
       <c r="W63" t="inlineStr"/>
       <c r="X63" t="n">
         <v>78.34001199635642</v>

</xml_diff>

<commit_message>
Fix systemic operating_expenses bug: compute from components
The extractor was matching "Other operating expenses" (a subtotal) as
operating_expenses, which excluded personnel expenses and depreciation.
This affected 93 of 128 bank-years, making operating_expenses appear
2-5x smaller than reality.

Fix: extract all 3 components (personnel, other operating, depreciation)
separately and compute operating_expenses = personnel + other + depreciation.

Also extracted other_operating_expenses and depreciation as new columns
for transparency, and fixed sign-flip bugs in NIMB/CZBIL FY2025.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/DATA/02_bank_ratios.xlsx
+++ b/DATA/02_bank_ratios.xlsx
@@ -626,7 +626,7 @@
         <v>5.876809114756854</v>
       </c>
       <c r="M3" t="n">
-        <v>11.46611327630713</v>
+        <v>47.77810396315229</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
@@ -688,7 +688,7 @@
         <v>-36.90305425310556</v>
       </c>
       <c r="M4" t="n">
-        <v>8.931800449298304</v>
+        <v>52.92852798489505</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -756,7 +756,7 @@
         <v>-40.54147553430947</v>
       </c>
       <c r="M5" t="n">
-        <v>10.37049612651778</v>
+        <v>53.15492470717141</v>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
@@ -824,7 +824,7 @@
         <v>118.9412200300738</v>
       </c>
       <c r="M6" t="n">
-        <v>8.137456752218442</v>
+        <v>46.06482011868795</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
@@ -892,7 +892,7 @@
         <v>28.81563007982773</v>
       </c>
       <c r="M7" t="n">
-        <v>8.688474668632699</v>
+        <v>50.72321709503512</v>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
@@ -996,7 +996,7 @@
         <v>18.19059355103718</v>
       </c>
       <c r="M9" t="n">
-        <v>13.30664365507127</v>
+        <v>43.39713392465588</v>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
@@ -1044,7 +1044,7 @@
         <v>34.53003631813996</v>
       </c>
       <c r="M10" t="n">
-        <v>11.73528379521873</v>
+        <v>47.07958237608116</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
         <v>-21.77793245745963</v>
       </c>
       <c r="M12" t="n">
-        <v>17.12523206585267</v>
+        <v>52.71881313255339</v>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
@@ -1254,7 +1254,7 @@
         <v>-4.914783987316684</v>
       </c>
       <c r="M14" t="n">
-        <v>18.10161771108953</v>
+        <v>58.87095153565328</v>
       </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -1310,7 +1310,7 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>18.10161771108953</v>
+        <v>58.87095153565328</v>
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
@@ -1412,7 +1412,7 @@
         <v>-28.29221377928973</v>
       </c>
       <c r="M17" t="n">
-        <v>13.06901113394103</v>
+        <v>42.71589350982513</v>
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
@@ -1474,7 +1474,7 @@
         <v>11.15477127370672</v>
       </c>
       <c r="M18" t="n">
-        <v>12.83273148724629</v>
+        <v>47.93025609588669</v>
       </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
@@ -1542,7 +1542,7 @@
         <v>-7.072661185375018</v>
       </c>
       <c r="M19" t="n">
-        <v>13.05024120757163</v>
+        <v>45.13403153785382</v>
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
@@ -1610,7 +1610,7 @@
         <v>-29.13626217967978</v>
       </c>
       <c r="M20" t="n">
-        <v>13.44919107884023</v>
+        <v>46.52093757483778</v>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
@@ -1678,7 +1678,7 @@
         <v>-2.547833395167831</v>
       </c>
       <c r="M21" t="n">
-        <v>13.13713785223931</v>
+        <v>42.91105391665157</v>
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
@@ -1782,7 +1782,7 @@
         <v>-29.61959113598066</v>
       </c>
       <c r="M23" t="n">
-        <v>13.65077271013946</v>
+        <v>47.02657369016208</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
@@ -1844,7 +1844,7 @@
         <v>40.00474324370109</v>
       </c>
       <c r="M24" t="n">
-        <v>8.700059349970914</v>
+        <v>43.05634721495855</v>
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
@@ -1912,7 +1912,7 @@
         <v>35.60216181334192</v>
       </c>
       <c r="M25" t="n">
-        <v>8.404668106482479</v>
+        <v>36.23589704974666</v>
       </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
@@ -1980,7 +1980,7 @@
         <v>10.1456818911877</v>
       </c>
       <c r="M26" t="n">
-        <v>8.596304447539735</v>
+        <v>33.95546568926557</v>
       </c>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
@@ -2048,7 +2048,7 @@
         <v>30.69401576461628</v>
       </c>
       <c r="M27" t="n">
-        <v>9.047393967389453</v>
+        <v>32.68493601966587</v>
       </c>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
@@ -2152,7 +2152,7 @@
         <v>43.19824248966877</v>
       </c>
       <c r="M29" t="n">
-        <v>11.45880226593813</v>
+        <v>40.73425432394212</v>
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
@@ -2214,7 +2214,7 @@
         <v>19.06461952150584</v>
       </c>
       <c r="M30" t="n">
-        <v>11.09647118012841</v>
+        <v>41.29728535798977</v>
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
@@ -2282,7 +2282,7 @@
         <v>34.98816346118944</v>
       </c>
       <c r="M31" t="n">
-        <v>9.444236571236917</v>
+        <v>34.75088872091167</v>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
@@ -2350,7 +2350,7 @@
         <v>-8.319092489797375</v>
       </c>
       <c r="M32" t="n">
-        <v>10.86960205636409</v>
+        <v>38.82244202435081</v>
       </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
@@ -2418,7 +2418,7 @@
         <v>-17.28975388801538</v>
       </c>
       <c r="M33" t="n">
-        <v>11.73603486630301</v>
+        <v>37.83394833774684</v>
       </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
@@ -2580,7 +2580,7 @@
         <v>-21.0456810132661</v>
       </c>
       <c r="M36" t="n">
-        <v>11.53194917315175</v>
+        <v>41.67740758754864</v>
       </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
@@ -2868,7 +2868,7 @@
         <v>70.10901934381231</v>
       </c>
       <c r="M41" t="n">
-        <v>13.25012476788677</v>
+        <v>47.82873902754486</v>
       </c>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
@@ -2930,7 +2930,7 @@
         <v>30.90631390398482</v>
       </c>
       <c r="M42" t="n">
-        <v>8.605669700648267</v>
+        <v>44.72381868643876</v>
       </c>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
@@ -2998,7 +2998,7 @@
         <v>-79.92410293781325</v>
       </c>
       <c r="M43" t="n">
-        <v>7.811111927999461</v>
+        <v>30.48190796527409</v>
       </c>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
         <v>-99.10990114303367</v>
       </c>
       <c r="M44" t="n">
-        <v>8.159766272966072</v>
+        <v>42.68781689035686</v>
       </c>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
@@ -3134,7 +3134,7 @@
         <v>39372.88503253796</v>
       </c>
       <c r="M45" t="n">
-        <v>6.920814899546005</v>
+        <v>40.51199090168369</v>
       </c>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
@@ -3238,7 +3238,7 @@
         <v>11.63331089936595</v>
       </c>
       <c r="M47" t="n">
-        <v>13.9939057193261</v>
+        <v>48.5904184590524</v>
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
@@ -3300,7 +3300,7 @@
         <v>24.49928923186271</v>
       </c>
       <c r="M48" t="n">
-        <v>9.728072537150103</v>
+        <v>47.5302455250519</v>
       </c>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
@@ -3368,7 +3368,7 @@
         <v>16.48630601332442</v>
       </c>
       <c r="M49" t="n">
-        <v>11.12126133441602</v>
+        <v>41.30816077953715</v>
       </c>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
@@ -3436,7 +3436,7 @@
         <v>27.79314207698098</v>
       </c>
       <c r="M50" t="n">
-        <v>9.064846215013363</v>
+        <v>46.42916048160977</v>
       </c>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
@@ -3504,7 +3504,7 @@
         <v>39.0928577787822</v>
       </c>
       <c r="M51" t="n">
-        <v>9.800927812409297</v>
+        <v>48.52872736877118</v>
       </c>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
@@ -3670,7 +3670,7 @@
         <v>4.92637498678048</v>
       </c>
       <c r="M54" t="n">
-        <v>17.25799952147688</v>
+        <v>53.46441299064362</v>
       </c>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
@@ -3738,7 +3738,7 @@
         <v>-3.62432262578114</v>
       </c>
       <c r="M55" t="n">
-        <v>11.67830701391599</v>
+        <v>48.61160462041206</v>
       </c>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
@@ -3874,7 +3874,7 @@
         <v>80.21814006888634</v>
       </c>
       <c r="M57" t="n">
-        <v>11.42235847040656</v>
+        <v>50.21563918303056</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
@@ -3990,7 +3990,7 @@
         <v>30.73162703133483</v>
       </c>
       <c r="M59" t="n">
-        <v>9.029001728182235</v>
+        <v>39.50470211369981</v>
       </c>
       <c r="N59" t="n">
         <v>134.3796029547553</v>
@@ -4064,7 +4064,7 @@
         <v>-5.997283298914413</v>
       </c>
       <c r="M60" t="n">
-        <v>8.923427439844437</v>
+        <v>35.49812301221021</v>
       </c>
       <c r="N60" t="n">
         <v>187.8380760626398</v>
@@ -4142,7 +4142,7 @@
         <v>50.49130408221762</v>
       </c>
       <c r="M61" t="n">
-        <v>7.111801675652793</v>
+        <v>30.50353319904541</v>
       </c>
       <c r="N61" t="n">
         <v>200.1678660565724</v>
@@ -4220,7 +4220,7 @@
         <v>-3.24483913978898</v>
       </c>
       <c r="M62" t="n">
-        <v>8.297967245915586</v>
+        <v>34.59143060829014</v>
       </c>
       <c r="N62" t="n">
         <v>231.7054450915142</v>
@@ -4298,7 +4298,7 @@
         <v>-4.437068246327714</v>
       </c>
       <c r="M63" t="n">
-        <v>8.378398964125218</v>
+        <v>36.03663645365221</v>
       </c>
       <c r="N63" t="n">
         <v>265.1071482098251</v>
@@ -4416,7 +4416,7 @@
         <v>26.93397459803077</v>
       </c>
       <c r="M65" t="n">
-        <v>9.928929051166199</v>
+        <v>40.83184760043962</v>
       </c>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
@@ -4478,7 +4478,7 @@
         <v>-1.2815620536061</v>
       </c>
       <c r="M66" t="n">
-        <v>9.76138371669397</v>
+        <v>40.14481044280818</v>
       </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
@@ -4546,7 +4546,7 @@
         <v>17.59325141621739</v>
       </c>
       <c r="M67" t="n">
-        <v>8.627700832589081</v>
+        <v>48.73201209498687</v>
       </c>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
@@ -4614,7 +4614,7 @@
         <v>0</v>
       </c>
       <c r="M68" t="n">
-        <v>8.627700832589081</v>
+        <v>48.73201209498687</v>
       </c>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
@@ -4682,7 +4682,7 @@
         <v>-10.4593929450369</v>
       </c>
       <c r="M69" t="n">
-        <v>9.017266734026272</v>
+        <v>44.12520883144426</v>
       </c>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
@@ -4786,7 +4786,7 @@
         <v>5.176308842228927</v>
       </c>
       <c r="M71" t="n">
-        <v>14.21857839756851</v>
+        <v>46.9468583461698</v>
       </c>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
@@ -4848,7 +4848,7 @@
         <v>29.33478166146559</v>
       </c>
       <c r="M72" t="n">
-        <v>15.20924160051876</v>
+        <v>50.56631001800612</v>
       </c>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
@@ -4916,7 +4916,7 @@
         <v>5.452996846922731</v>
       </c>
       <c r="M73" t="n">
-        <v>13.48285819051542</v>
+        <v>51.69428304665492</v>
       </c>
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
@@ -4984,7 +4984,7 @@
         <v>-84.217406075005</v>
       </c>
       <c r="M74" t="n">
-        <v>15.5345328624826</v>
+        <v>55.39234337645781</v>
       </c>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
@@ -5052,7 +5052,7 @@
         <v>-650.6999287241624</v>
       </c>
       <c r="M75" t="n">
-        <v>15.45608050134878</v>
+        <v>55.15145483124782</v>
       </c>
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
@@ -5218,7 +5218,7 @@
         <v>6.715824437069529</v>
       </c>
       <c r="M78" t="n">
-        <v>8.956583718119557</v>
+        <v>38.23471443180762</v>
       </c>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
@@ -5286,7 +5286,7 @@
         <v>-2.021539919949444</v>
       </c>
       <c r="M79" t="n">
-        <v>8.017160767765599</v>
+        <v>33.3995776165194</v>
       </c>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
@@ -5354,7 +5354,7 @@
         <v>10.42939344178584</v>
       </c>
       <c r="M80" t="n">
-        <v>8.813990571972267</v>
+        <v>35.27081666435974</v>
       </c>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
@@ -5422,7 +5422,7 @@
         <v>5.436748124189239</v>
       </c>
       <c r="M81" t="n">
-        <v>9.124950148647669</v>
+        <v>37.0831747153941</v>
       </c>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
@@ -5526,7 +5526,7 @@
         <v>58.28477679561883</v>
       </c>
       <c r="M83" t="n">
-        <v>11.51171194494334</v>
+        <v>43.32219579416318</v>
       </c>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
@@ -5588,7 +5588,7 @@
         <v>21.39450475273601</v>
       </c>
       <c r="M84" t="n">
-        <v>12.73919957283072</v>
+        <v>45.87608343852533</v>
       </c>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
@@ -5656,7 +5656,7 @@
         <v>-2.082592697252272</v>
       </c>
       <c r="M85" t="n">
-        <v>11.53977589002638</v>
+        <v>40.66516614632494</v>
       </c>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
@@ -5724,7 +5724,7 @@
         <v>-30.35329164791858</v>
       </c>
       <c r="M86" t="n">
-        <v>10.8047119204523</v>
+        <v>43.70687105416027</v>
       </c>
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
@@ -5792,7 +5792,7 @@
         <v>27.18944929602565</v>
       </c>
       <c r="M87" t="n">
-        <v>10.18878186635699</v>
+        <v>41.40145821772573</v>
       </c>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
@@ -5896,7 +5896,7 @@
         <v>45.16673477001794</v>
       </c>
       <c r="M89" t="n">
-        <v>7.807427581968362</v>
+        <v>30.4492353359702</v>
       </c>
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
@@ -5958,7 +5958,7 @@
         <v>-14.71851670542161</v>
       </c>
       <c r="M90" t="n">
-        <v>6.158108265052727</v>
+        <v>32.25728576592377</v>
       </c>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
@@ -6026,7 +6026,7 @@
         <v>-63.12254694439861</v>
       </c>
       <c r="M91" t="n">
-        <v>6.130846678892434</v>
+        <v>28.45928622115785</v>
       </c>
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
@@ -6094,7 +6094,7 @@
         <v>241.2676330382332</v>
       </c>
       <c r="M92" t="n">
-        <v>5.373338309211509</v>
+        <v>29.33127654663207</v>
       </c>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
@@ -6162,7 +6162,7 @@
         <v>-8.755405671215454</v>
       </c>
       <c r="M93" t="n">
-        <v>4.915645037804787</v>
+        <v>27.94246451827461</v>
       </c>
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
@@ -6266,7 +6266,7 @@
         <v>44.10232791827162</v>
       </c>
       <c r="M95" t="n">
-        <v>17.65784390094235</v>
+        <v>59.49937966092102</v>
       </c>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
@@ -6328,7 +6328,7 @@
         <v>10.52665221661138</v>
       </c>
       <c r="M96" t="n">
-        <v>13.72716743350795</v>
+        <v>56.3961735859482</v>
       </c>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
@@ -6396,7 +6396,7 @@
         <v>-85.2672421951399</v>
       </c>
       <c r="M97" t="n">
-        <v>12.20616650366004</v>
+        <v>44.37750525007465</v>
       </c>
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
@@ -6464,7 +6464,7 @@
         <v>82.30675897509099</v>
       </c>
       <c r="M98" t="n">
-        <v>10.75972178659667</v>
+        <v>45.86834387088609</v>
       </c>
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
@@ -6532,7 +6532,7 @@
         <v>70.75715460204361</v>
       </c>
       <c r="M99" t="n">
-        <v>13.86107335639288</v>
+        <v>59.68183886128617</v>
       </c>
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
@@ -6636,7 +6636,7 @@
         <v>-21.78661829612639</v>
       </c>
       <c r="M101" t="n">
-        <v>12.69126783101071</v>
+        <v>46.31399033106985</v>
       </c>
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
@@ -6766,7 +6766,7 @@
         <v>-16.25248671036753</v>
       </c>
       <c r="M103" t="n">
-        <v>8.785692913759696</v>
+        <v>42.94055269704916</v>
       </c>
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
@@ -6834,7 +6834,7 @@
         <v>-29.00201105384229</v>
       </c>
       <c r="M104" t="n">
-        <v>11.6543639333868</v>
+        <v>54.64007359119123</v>
       </c>
       <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
@@ -6902,7 +6902,7 @@
         <v>11.10806395373893</v>
       </c>
       <c r="M105" t="n">
-        <v>10.60924499706164</v>
+        <v>52.24049673687792</v>
       </c>
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
@@ -7006,7 +7006,7 @@
         <v>30.48877979575064</v>
       </c>
       <c r="M107" t="n">
-        <v>11.27863103883937</v>
+        <v>38.81909051061014</v>
       </c>
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr"/>
@@ -7068,7 +7068,7 @@
         <v>-9.694454271686336</v>
       </c>
       <c r="M108" t="n">
-        <v>10.37248951025756</v>
+        <v>41.80556246579432</v>
       </c>
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr"/>
@@ -7136,7 +7136,7 @@
         <v>24.4931012077664</v>
       </c>
       <c r="M109" t="n">
-        <v>9.209336365299666</v>
+        <v>36.96345957813848</v>
       </c>
       <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr"/>
@@ -7204,7 +7204,7 @@
         <v>-7.995655827983061</v>
       </c>
       <c r="M110" t="n">
-        <v>9.456894475112341</v>
+        <v>38.14867644592088</v>
       </c>
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr"/>
@@ -7272,7 +7272,7 @@
         <v>7.300286972770964</v>
       </c>
       <c r="M111" t="n">
-        <v>9.091352938578035</v>
+        <v>36.4715441861979</v>
       </c>
       <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr"/>
@@ -7376,7 +7376,7 @@
         <v>-37.57216444746817</v>
       </c>
       <c r="M113" t="n">
-        <v>17.53516926688882</v>
+        <v>59.03206414722811</v>
       </c>
       <c r="N113" t="inlineStr"/>
       <c r="O113" t="inlineStr"/>
@@ -7438,7 +7438,7 @@
         <v>70.0408934279902</v>
       </c>
       <c r="M114" t="n">
-        <v>10.64295613286285</v>
+        <v>48.35683996253685</v>
       </c>
       <c r="N114" t="inlineStr"/>
       <c r="O114" t="inlineStr"/>
@@ -7506,7 +7506,7 @@
         <v>20.0938772271426</v>
       </c>
       <c r="M115" t="n">
-        <v>9.568118360491242</v>
+        <v>41.06583884126257</v>
       </c>
       <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr"/>
@@ -7574,7 +7574,7 @@
         <v>1.639635884951018</v>
       </c>
       <c r="M116" t="n">
-        <v>10.78420818609441</v>
+        <v>45.63416099162981</v>
       </c>
       <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr"/>
@@ -7642,7 +7642,7 @@
         <v>-9.441585782364969</v>
       </c>
       <c r="M117" t="n">
-        <v>11.19306131027884</v>
+        <v>44.50326959737433</v>
       </c>
       <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr"/>
@@ -7746,7 +7746,7 @@
         <v>33.17860991504984</v>
       </c>
       <c r="M119" t="n">
-        <v>11.01453179909297</v>
+        <v>41.39305810592687</v>
       </c>
       <c r="N119" t="inlineStr"/>
       <c r="O119" t="inlineStr"/>
@@ -7808,7 +7808,7 @@
         <v>1.66840057026163</v>
       </c>
       <c r="M120" t="n">
-        <v>9.416092184118007</v>
+        <v>44.56282266659235</v>
       </c>
       <c r="N120" t="inlineStr"/>
       <c r="O120" t="inlineStr"/>
@@ -7876,7 +7876,7 @@
         <v>9.106413180543393</v>
       </c>
       <c r="M121" t="n">
-        <v>9.121286747270645</v>
+        <v>41.93272573802746</v>
       </c>
       <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr"/>
@@ -7944,7 +7944,7 @@
         <v>-2.739068514606358</v>
       </c>
       <c r="M122" t="n">
-        <v>9.878724705080534</v>
+        <v>44.51785553205777</v>
       </c>
       <c r="N122" t="inlineStr"/>
       <c r="O122" t="inlineStr"/>
@@ -8012,7 +8012,7 @@
         <v>9.303805482414141</v>
       </c>
       <c r="M123" t="n">
-        <v>9.551811211935684</v>
+        <v>43.07736162118505</v>
       </c>
       <c r="N123" t="inlineStr"/>
       <c r="O123" t="inlineStr"/>
@@ -8178,7 +8178,7 @@
         <v>61.27148208515627</v>
       </c>
       <c r="M126" t="n">
-        <v>10.16355205897849</v>
+        <v>36.72487142516973</v>
       </c>
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr"/>
@@ -8246,7 +8246,7 @@
         <v>53.6098194536178</v>
       </c>
       <c r="M127" t="n">
-        <v>7.281177678178653</v>
+        <v>28.9778197142511</v>
       </c>
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr"/>
@@ -8314,7 +8314,7 @@
         <v>-5.484614740876048</v>
       </c>
       <c r="M128" t="n">
-        <v>7.650415296405192</v>
+        <v>31.81906186989869</v>
       </c>
       <c r="N128" t="inlineStr"/>
       <c r="O128" t="inlineStr"/>
@@ -8382,7 +8382,7 @@
         <v>-8.021018114537126</v>
       </c>
       <c r="M129" t="n">
-        <v>8.126442078814122</v>
+        <v>33.81502758296563</v>
       </c>
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="inlineStr"/>

</xml_diff>